<commit_message>
Updated lib and simplified LCD code
</commit_message>
<xml_diff>
--- a/INFO_and_DATASHEETS/suminis_neapibreztumas.xlsx
+++ b/INFO_and_DATASHEETS/suminis_neapibreztumas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Linas\Desktop\univero darbai\Iterptines_sistemos\Inzinerinis_projektas\INFO_and_DATASHEETS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03BEE6E1-EA07-429E-8D56-E16B7C4FC69D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{691CDD05-ACC7-4661-ABDA-261F8024A3AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
   <si>
     <t>u</t>
   </si>
@@ -79,13 +79,19 @@
   <si>
     <t>V</t>
   </si>
+  <si>
+    <t>SUMINIS</t>
+  </si>
+  <si>
+    <t>SAKNIS</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -116,15 +122,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -868,7 +873,608 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$24:$B$57</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.1000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.3</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.4</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.7</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.9</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.2000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.2999999999999998</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2.7</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2.8</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2.9</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>3.1</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3.2</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>3.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$J$24:$J$57</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>48.205452136713099</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>96.410904273426198</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>144.6163564101393</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>192.8218085468524</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>241.02726068356549</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>289.23271282027861</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>337.43816495699161</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>385.64361709370479</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>433.84906923041785</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>482.05452136713097</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>530.25997350384409</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>578.46542564055721</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>626.67087777727033</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>674.87632991398323</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>723.08178205069646</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>771.28723418740958</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>819.49268632412259</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>867.69813846083571</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>915.90359059754871</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>964.10904273426195</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1012.3144948709751</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1060.5199470076882</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1108.7253991444011</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1156.9308512811144</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1205.1363034178273</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1253.3417555545407</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1301.5472076912538</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1349.7526598279665</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1397.9581119646798</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1446.1635641013929</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>1494.369016238106</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>1542.5744683748192</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1590.7799205115321</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5D4B-4840-8BA7-A192BC2B3F03}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="479774927"/>
+        <c:axId val="479758607"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="479774927"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="lt-LT"/>
+                  <a:t>Įtampa, V</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="lt-LT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="lt-LT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="479758607"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="479758607"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="lt-LT"/>
+                  <a:t>Apšviestumo neapibrėžtumas, lux</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="lt-LT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="lt-LT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="479774927"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="lt-LT"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1424,20 +2030,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>488576</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>62752</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>22411</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>116541</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>1304364</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>116540</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>49305</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>170329</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1457,6 +2579,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>243429</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>82998</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2A12358A-D8C3-FCEC-A0E0-EB72B32E71AA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1867,7 +3025,7 @@
         <v>0.1</v>
       </c>
       <c r="D12" s="1">
-        <f t="shared" ref="D12:D14" si="0">1/($B$4*$B$5)</f>
+        <f t="shared" ref="D12:D13" si="0">1/($B$4*$B$5)</f>
         <v>3048.7804878048778</v>
       </c>
       <c r="E12" s="1">
@@ -1879,11 +3037,11 @@
         <v>-762195121951.21948</v>
       </c>
       <c r="H12" s="1">
-        <f t="shared" ref="H12:H13" si="2">D12*$E$4</f>
+        <f t="shared" ref="H12" si="2">D12*$E$4</f>
         <v>0.70731707317073167</v>
       </c>
       <c r="I12" s="1">
-        <f t="shared" ref="I12:I13" si="3">E12*$E$5</f>
+        <f t="shared" ref="I12" si="3">E12*$E$5</f>
         <v>-15.243902439024389</v>
       </c>
       <c r="J12" s="1">
@@ -1891,7 +3049,7 @@
         <v>-45.731707317073166</v>
       </c>
       <c r="L12" s="1">
-        <f t="shared" ref="L12:L13" si="5">H12^2+I12^2+J12^2</f>
+        <f t="shared" ref="L12" si="5">H12^2+I12^2+J12^2</f>
         <v>2324.2659131469359</v>
       </c>
       <c r="N12" s="1">
@@ -1976,34 +3134,32 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E18" s="1">
         <f>-(B16/($B$5*$B$4^2))</f>
         <v>-3.7180249851278997E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E22" s="4" t="s">
         <v>6</v>
       </c>
       <c r="F22" s="4"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>13</v>
       </c>
@@ -2019,8 +3175,14 @@
       <c r="H23" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B24" s="3">
         <v>0</v>
       </c>
@@ -2048,8 +3210,16 @@
         <f>F24*F24</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I24" s="1">
+        <f>G24+H24</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="1">
+        <f>SQRT(I24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B25" s="3">
         <v>0.1</v>
       </c>
@@ -2077,8 +3247,16 @@
         <f t="shared" ref="H25:H57" si="13">F25*F25</f>
         <v>2091.3890541344435</v>
       </c>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I25" s="1">
+        <f t="shared" ref="I25:I57" si="14">G25+H25</f>
+        <v>2323.7656157049373</v>
+      </c>
+      <c r="J25" s="1">
+        <f t="shared" ref="J25:J57" si="15">SQRT(I25)</f>
+        <v>48.205452136713099</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B26" s="3">
         <v>0.2</v>
       </c>
@@ -2106,8 +3284,16 @@
         <f t="shared" si="13"/>
         <v>8365.5562165377742</v>
       </c>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I26" s="1">
+        <f t="shared" si="14"/>
+        <v>9295.0624628197493</v>
+      </c>
+      <c r="J26" s="1">
+        <f t="shared" si="15"/>
+        <v>96.410904273426198</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B27" s="3">
         <v>0.3</v>
       </c>
@@ -2135,8 +3321,16 @@
         <f t="shared" si="13"/>
         <v>18822.501487209993</v>
       </c>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I27" s="1">
+        <f t="shared" si="14"/>
+        <v>20913.890541344437</v>
+      </c>
+      <c r="J27" s="1">
+        <f t="shared" si="15"/>
+        <v>144.6163564101393</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B28" s="3">
         <v>0.4</v>
       </c>
@@ -2164,8 +3358,16 @@
         <f t="shared" si="13"/>
         <v>33462.224866151097</v>
       </c>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I28" s="1">
+        <f t="shared" si="14"/>
+        <v>37180.249851278997</v>
+      </c>
+      <c r="J28" s="1">
+        <f t="shared" si="15"/>
+        <v>192.8218085468524</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B29" s="3">
         <v>0.5</v>
       </c>
@@ -2193,8 +3395,16 @@
         <f t="shared" si="13"/>
         <v>52284.726353361082</v>
       </c>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I29" s="1">
+        <f t="shared" si="14"/>
+        <v>58094.140392623427</v>
+      </c>
+      <c r="J29" s="1">
+        <f t="shared" si="15"/>
+        <v>241.02726068356549</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B30" s="3">
         <v>0.6</v>
       </c>
@@ -2222,8 +3432,16 @@
         <f t="shared" si="13"/>
         <v>75290.005948839971</v>
       </c>
-    </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I30" s="1">
+        <f t="shared" si="14"/>
+        <v>83655.562165377749</v>
+      </c>
+      <c r="J30" s="1">
+        <f t="shared" si="15"/>
+        <v>289.23271282027861</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B31" s="3">
         <v>0.7</v>
       </c>
@@ -2251,8 +3469,16 @@
         <f t="shared" si="13"/>
         <v>102478.06365258771</v>
       </c>
-    </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I31" s="1">
+        <f t="shared" si="14"/>
+        <v>113864.51516954189</v>
+      </c>
+      <c r="J31" s="1">
+        <f t="shared" si="15"/>
+        <v>337.43816495699161</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B32" s="3">
         <v>0.8</v>
       </c>
@@ -2280,8 +3506,16 @@
         <f t="shared" si="13"/>
         <v>133848.89946460439</v>
       </c>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I32" s="1">
+        <f t="shared" si="14"/>
+        <v>148720.99940511599</v>
+      </c>
+      <c r="J32" s="1">
+        <f t="shared" si="15"/>
+        <v>385.64361709370479</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B33" s="3">
         <v>0.9</v>
       </c>
@@ -2309,8 +3543,16 @@
         <f t="shared" si="13"/>
         <v>169402.51338488993</v>
       </c>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I33" s="1">
+        <f t="shared" si="14"/>
+        <v>188225.01487209991</v>
+      </c>
+      <c r="J33" s="1">
+        <f t="shared" si="15"/>
+        <v>433.84906923041785</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B34" s="3">
         <v>1</v>
       </c>
@@ -2338,8 +3580,16 @@
         <f t="shared" si="13"/>
         <v>209138.90541344433</v>
       </c>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I34" s="1">
+        <f t="shared" si="14"/>
+        <v>232376.56157049371</v>
+      </c>
+      <c r="J34" s="1">
+        <f t="shared" si="15"/>
+        <v>482.05452136713097</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B35" s="3">
         <v>1.1000000000000001</v>
       </c>
@@ -2367,8 +3617,16 @@
         <f t="shared" si="13"/>
         <v>253058.07555026771</v>
       </c>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I35" s="1">
+        <f t="shared" si="14"/>
+        <v>281175.63950029743</v>
+      </c>
+      <c r="J35" s="1">
+        <f t="shared" si="15"/>
+        <v>530.25997350384409</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B36" s="3">
         <v>1.2</v>
       </c>
@@ -2396,8 +3654,16 @@
         <f t="shared" si="13"/>
         <v>301160.02379535988</v>
       </c>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I36" s="1">
+        <f t="shared" si="14"/>
+        <v>334622.248661511</v>
+      </c>
+      <c r="J36" s="1">
+        <f t="shared" si="15"/>
+        <v>578.46542564055721</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B37" s="3">
         <v>1.3</v>
       </c>
@@ -2425,8 +3691,16 @@
         <f t="shared" si="13"/>
         <v>353444.75014872098</v>
       </c>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I37" s="1">
+        <f t="shared" si="14"/>
+        <v>392716.38905413443</v>
+      </c>
+      <c r="J37" s="1">
+        <f t="shared" si="15"/>
+        <v>626.67087777727033</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B38" s="3">
         <v>1.4</v>
       </c>
@@ -2454,8 +3728,16 @@
         <f t="shared" si="13"/>
         <v>409912.25461035082</v>
       </c>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I38" s="1">
+        <f t="shared" si="14"/>
+        <v>455458.06067816756</v>
+      </c>
+      <c r="J38" s="1">
+        <f t="shared" si="15"/>
+        <v>674.87632991398323</v>
+      </c>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B39" s="3">
         <v>1.5</v>
       </c>
@@ -2483,8 +3765,16 @@
         <f t="shared" si="13"/>
         <v>470562.53718024975</v>
       </c>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I39" s="1">
+        <f t="shared" si="14"/>
+        <v>522847.26353361085</v>
+      </c>
+      <c r="J39" s="1">
+        <f t="shared" si="15"/>
+        <v>723.08178205069646</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B40" s="3">
         <v>1.6</v>
       </c>
@@ -2512,8 +3802,16 @@
         <f t="shared" si="13"/>
         <v>535395.59785841755</v>
       </c>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I40" s="1">
+        <f t="shared" si="14"/>
+        <v>594883.99762046395</v>
+      </c>
+      <c r="J40" s="1">
+        <f t="shared" si="15"/>
+        <v>771.28723418740958</v>
+      </c>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B41" s="3">
         <v>1.7</v>
       </c>
@@ -2541,8 +3839,16 @@
         <f t="shared" si="13"/>
         <v>604411.43664485414</v>
       </c>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I41" s="1">
+        <f t="shared" si="14"/>
+        <v>671568.26293872681</v>
+      </c>
+      <c r="J41" s="1">
+        <f t="shared" si="15"/>
+        <v>819.49268632412259</v>
+      </c>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B42" s="3">
         <v>1.8</v>
       </c>
@@ -2570,8 +3876,16 @@
         <f t="shared" si="13"/>
         <v>677610.05353955971</v>
       </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I42" s="1">
+        <f t="shared" si="14"/>
+        <v>752900.05948839965</v>
+      </c>
+      <c r="J42" s="1">
+        <f t="shared" si="15"/>
+        <v>867.69813846083571</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B43" s="3">
         <v>1.9</v>
       </c>
@@ -2599,8 +3913,16 @@
         <f t="shared" si="13"/>
         <v>754991.44854253391</v>
       </c>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I43" s="1">
+        <f t="shared" si="14"/>
+        <v>838879.38726948213</v>
+      </c>
+      <c r="J43" s="1">
+        <f t="shared" si="15"/>
+        <v>915.90359059754871</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B44" s="3">
         <v>2</v>
       </c>
@@ -2628,8 +3950,16 @@
         <f t="shared" si="13"/>
         <v>836555.62165377731</v>
       </c>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I44" s="1">
+        <f t="shared" si="14"/>
+        <v>929506.24628197483</v>
+      </c>
+      <c r="J44" s="1">
+        <f t="shared" si="15"/>
+        <v>964.10904273426195</v>
+      </c>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B45" s="3">
         <v>2.1</v>
       </c>
@@ -2657,8 +3987,16 @@
         <f t="shared" si="13"/>
         <v>922302.5728732897</v>
       </c>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I45" s="1">
+        <f t="shared" si="14"/>
+        <v>1024780.6365258774</v>
+      </c>
+      <c r="J45" s="1">
+        <f t="shared" si="15"/>
+        <v>1012.3144948709751</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B46" s="3">
         <v>2.2000000000000002</v>
       </c>
@@ -2686,8 +4024,16 @@
         <f t="shared" si="13"/>
         <v>1012232.3022010708</v>
       </c>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I46" s="1">
+        <f t="shared" si="14"/>
+        <v>1124702.5580011897</v>
+      </c>
+      <c r="J46" s="1">
+        <f t="shared" si="15"/>
+        <v>1060.5199470076882</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B47" s="3">
         <v>2.2999999999999998</v>
       </c>
@@ -2715,8 +4061,16 @@
         <f t="shared" si="13"/>
         <v>1106344.8096371202</v>
       </c>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I47" s="1">
+        <f t="shared" si="14"/>
+        <v>1229272.0107079113</v>
+      </c>
+      <c r="J47" s="1">
+        <f t="shared" si="15"/>
+        <v>1108.7253991444011</v>
+      </c>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B48" s="3">
         <v>2.4</v>
       </c>
@@ -2744,8 +4098,16 @@
         <f t="shared" si="13"/>
         <v>1204640.0951814395</v>
       </c>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I48" s="1">
+        <f t="shared" si="14"/>
+        <v>1338488.994646044</v>
+      </c>
+      <c r="J48" s="1">
+        <f t="shared" si="15"/>
+        <v>1156.9308512811144</v>
+      </c>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B49" s="3">
         <v>2.5</v>
       </c>
@@ -2773,8 +4135,16 @@
         <f t="shared" si="13"/>
         <v>1307118.1588340267</v>
       </c>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I49" s="1">
+        <f t="shared" si="14"/>
+        <v>1452353.5098155853</v>
+      </c>
+      <c r="J49" s="1">
+        <f t="shared" si="15"/>
+        <v>1205.1363034178273</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B50" s="3">
         <v>2.6</v>
       </c>
@@ -2802,8 +4172,16 @@
         <f t="shared" si="13"/>
         <v>1413779.0005948839</v>
       </c>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I50" s="1">
+        <f t="shared" si="14"/>
+        <v>1570865.5562165377</v>
+      </c>
+      <c r="J50" s="1">
+        <f t="shared" si="15"/>
+        <v>1253.3417555545407</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B51" s="3">
         <v>2.7</v>
       </c>
@@ -2831,8 +4209,16 @@
         <f t="shared" si="13"/>
         <v>1524622.6204640095</v>
       </c>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I51" s="1">
+        <f t="shared" si="14"/>
+        <v>1694025.1338488995</v>
+      </c>
+      <c r="J51" s="1">
+        <f t="shared" si="15"/>
+        <v>1301.5472076912538</v>
+      </c>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B52" s="3">
         <v>2.8</v>
       </c>
@@ -2860,8 +4246,16 @@
         <f t="shared" si="13"/>
         <v>1639649.0184414033</v>
       </c>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I52" s="1">
+        <f t="shared" si="14"/>
+        <v>1821832.2427126702</v>
+      </c>
+      <c r="J52" s="1">
+        <f t="shared" si="15"/>
+        <v>1349.7526598279665</v>
+      </c>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B53" s="3">
         <v>2.9</v>
       </c>
@@ -2889,8 +4283,16 @@
         <f t="shared" si="13"/>
         <v>1758858.1945270668</v>
       </c>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I53" s="1">
+        <f t="shared" si="14"/>
+        <v>1954286.882807852</v>
+      </c>
+      <c r="J53" s="1">
+        <f t="shared" si="15"/>
+        <v>1397.9581119646798</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B54" s="3">
         <v>3</v>
       </c>
@@ -2918,8 +4320,16 @@
         <f t="shared" si="13"/>
         <v>1882250.148720999</v>
       </c>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I54" s="1">
+        <f t="shared" si="14"/>
+        <v>2091389.0541344434</v>
+      </c>
+      <c r="J54" s="1">
+        <f t="shared" si="15"/>
+        <v>1446.1635641013929</v>
+      </c>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B55" s="3">
         <v>3.1</v>
       </c>
@@ -2947,8 +4357,16 @@
         <f t="shared" si="13"/>
         <v>2009824.8810232007</v>
       </c>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I55" s="1">
+        <f t="shared" si="14"/>
+        <v>2233138.7566924449</v>
+      </c>
+      <c r="J55" s="1">
+        <f t="shared" si="15"/>
+        <v>1494.369016238106</v>
+      </c>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B56" s="3">
         <v>3.2</v>
       </c>
@@ -2976,8 +4394,16 @@
         <f t="shared" si="13"/>
         <v>2141582.3914336702</v>
       </c>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I56" s="1">
+        <f t="shared" si="14"/>
+        <v>2379535.9904818558</v>
+      </c>
+      <c r="J56" s="1">
+        <f t="shared" si="15"/>
+        <v>1542.5744683748192</v>
+      </c>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B57" s="3">
         <v>3.3</v>
       </c>
@@ -3004,6 +4430,14 @@
       <c r="H57" s="1">
         <f t="shared" si="13"/>
         <v>2277522.6799524087</v>
+      </c>
+      <c r="I57" s="1">
+        <f t="shared" si="14"/>
+        <v>2530580.7555026761</v>
+      </c>
+      <c r="J57" s="1">
+        <f t="shared" si="15"/>
+        <v>1590.7799205115321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>